<commit_message>
data: update quran data from local excel file
</commit_message>
<xml_diff>
--- a/data/quran_data.xlsx
+++ b/data/quran_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdal_03\OneDrive\Documents\TRYING STUFF\برنامج الدورة القرآنية\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7822E906-7105-49C4-9CA6-97D3C0958213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4818C6D7-E453-40C7-A93F-DDA622FF400C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17436" yWindow="0" windowWidth="5700" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -1064,7 +1064,7 @@
         <v>49</v>
       </c>
       <c r="E20" s="1">
-        <v>260.5</v>
+        <v>260</v>
       </c>
       <c r="F20" s="1">
         <v>15</v>

</xml_diff>

<commit_message>
feat: add quran data file
</commit_message>
<xml_diff>
--- a/data/quran_data.xlsx
+++ b/data/quran_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdal_03\OneDrive\Documents\TRYING STUFF\برنامج الدورة القرآنية\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4818C6D7-E453-40C7-A93F-DDA622FF400C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3307709-2B59-4941-834E-E391D3B915C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17436" yWindow="0" windowWidth="5700" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -1064,7 +1064,7 @@
         <v>49</v>
       </c>
       <c r="E20" s="1">
-        <v>260</v>
+        <v>260.5</v>
       </c>
       <c r="F20" s="1">
         <v>15</v>

</xml_diff>

<commit_message>
feat: Add Quran data
</commit_message>
<xml_diff>
--- a/data/quran_data.xlsx
+++ b/data/quran_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdal_03\OneDrive\Documents\TRYING STUFF\برنامج الدورة القرآنية\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3307709-2B59-4941-834E-E391D3B915C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4032D404-7C45-409D-9DA4-2F6835F8CB8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -731,10 +731,10 @@
         <v>1</v>
       </c>
       <c r="E2" s="1">
-        <v>118.15</v>
+        <v>148.75</v>
       </c>
       <c r="F2" s="1">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="G2" s="1">
         <v>0</v>
@@ -754,13 +754,16 @@
         <v>39</v>
       </c>
       <c r="E3" s="1">
-        <v>194.75</v>
+        <v>242</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="J3" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -771,10 +774,10 @@
         <v>40</v>
       </c>
       <c r="E4" s="1">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="F4" s="1">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>10</v>
@@ -788,10 +791,10 @@
         <v>41</v>
       </c>
       <c r="E5" s="1">
-        <v>225.5</v>
+        <v>280.5</v>
       </c>
       <c r="F5" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>10</v>
@@ -808,13 +811,16 @@
         <v>42</v>
       </c>
       <c r="E6" s="1">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F6" s="1">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="J6" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -825,10 +831,10 @@
         <v>32</v>
       </c>
       <c r="E7" s="1">
-        <v>236.5</v>
+        <v>290</v>
       </c>
       <c r="F7" s="1">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>10</v>
@@ -845,13 +851,16 @@
         <v>43</v>
       </c>
       <c r="E8" s="1">
-        <v>74.5</v>
+        <v>121</v>
       </c>
       <c r="F8" s="1">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="J8" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -862,10 +871,10 @@
         <v>33</v>
       </c>
       <c r="E9" s="1">
-        <v>207</v>
+        <v>271</v>
       </c>
       <c r="F9" s="1">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>10</v>
@@ -882,16 +891,16 @@
         <v>44</v>
       </c>
       <c r="E10" s="1">
-        <v>68.5</v>
+        <v>122</v>
       </c>
       <c r="F10" s="1">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J10" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -902,13 +911,16 @@
         <v>46</v>
       </c>
       <c r="E11" s="1">
-        <v>12</v>
+        <v>31.5</v>
       </c>
       <c r="F11" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="J11" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -919,7 +931,7 @@
         <v>45</v>
       </c>
       <c r="E12" s="1">
-        <v>78.5</v>
+        <v>108</v>
       </c>
       <c r="F12" s="1">
         <v>3</v>
@@ -928,7 +940,7 @@
         <v>10</v>
       </c>
       <c r="J12" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -939,10 +951,10 @@
         <v>47</v>
       </c>
       <c r="E13" s="1">
-        <v>13.5</v>
+        <v>46</v>
       </c>
       <c r="F13" s="1">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>10</v>
@@ -956,16 +968,16 @@
         <v>34</v>
       </c>
       <c r="E14" s="1">
-        <v>134.5</v>
+        <v>184</v>
       </c>
       <c r="F14" s="1">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J14" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -976,13 +988,16 @@
         <v>35</v>
       </c>
       <c r="E15" s="1">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="F15" s="1">
         <v>1</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="J15" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -993,10 +1008,10 @@
         <v>32</v>
       </c>
       <c r="E16" s="1">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="F16" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>10</v>
@@ -1005,7 +1020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
@@ -1013,16 +1028,16 @@
         <v>36</v>
       </c>
       <c r="E17" s="1">
-        <v>146.5</v>
+        <v>183.5</v>
       </c>
       <c r="F17" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>26</v>
       </c>
@@ -1030,16 +1045,16 @@
         <v>37</v>
       </c>
       <c r="E18" s="1">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F18" s="1">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>27</v>
       </c>
@@ -1047,16 +1062,16 @@
         <v>48</v>
       </c>
       <c r="E19" s="1">
-        <v>20.5</v>
+        <v>25</v>
       </c>
       <c r="F19" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>28</v>
       </c>
@@ -1064,16 +1079,19 @@
         <v>49</v>
       </c>
       <c r="E20" s="1">
-        <v>260.5</v>
+        <v>305</v>
       </c>
       <c r="F20" s="1">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
@@ -1081,16 +1099,19 @@
         <v>50</v>
       </c>
       <c r="E21" s="1">
-        <v>166</v>
+        <v>234</v>
       </c>
       <c r="F21" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J21" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
         <v>30</v>
       </c>
@@ -1098,19 +1119,22 @@
         <v>38</v>
       </c>
       <c r="E22" s="1">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="F22" s="1">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="J22" s="1">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J1 C2 G2:H2 C3:D3 G3 C4:D4 G4 I3:J3 I4:J4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J1 C2 G2:H2 C3:D3 G3 C4:D4 G4 I3 I4:J4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>